<commit_message>
Home games: Turbo Tubs play at Equity Bank Park
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RVvxjtAiL6j1MniaJt2d1E
</commit_message>
<xml_diff>
--- a/Wichita home games 2026-27 (verified).xlsx
+++ b/Wichita home games 2026-27 (verified).xlsx
@@ -496,7 +496,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Turbo Tubs: MiLB data still lists the park as Equity Bank Park; confirm the venue name you want. Times are tentative until the team publishes its own.</t>
+          <t>Turbo Tubs: home games are at Equity Bank Park. Times are tentative until the team publishes its own.</t>
         </is>
       </c>
     </row>
@@ -4302,7 +4302,7 @@
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="52" customWidth="1" min="4" max="4"/>
-    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="56" customWidth="1" min="5" max="5"/>
     <col width="33" customWidth="1" min="6" max="6"/>
     <col width="39" customWidth="1" min="7" max="7"/>
   </cols>
@@ -4365,7 +4365,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -4400,7 +4400,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -4435,7 +4435,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -4470,7 +4470,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -4505,7 +4505,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -4540,7 +4540,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -4575,7 +4575,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -4610,7 +4610,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -4645,7 +4645,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -4680,7 +4680,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -4715,7 +4715,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -4750,7 +4750,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -4785,7 +4785,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -4820,7 +4820,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -4855,7 +4855,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -4890,7 +4890,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -4925,7 +4925,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -4960,7 +4960,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -4995,7 +4995,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -5030,7 +5030,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -5065,7 +5065,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -5100,7 +5100,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -5135,7 +5135,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -5170,7 +5170,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -5205,7 +5205,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -5240,7 +5240,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -5275,7 +5275,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -5310,7 +5310,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -5345,7 +5345,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -5380,7 +5380,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -5415,7 +5415,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -5450,7 +5450,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -5485,7 +5485,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -5520,7 +5520,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -5555,7 +5555,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -5590,7 +5590,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -5625,7 +5625,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -5660,7 +5660,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -5695,7 +5695,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -5730,7 +5730,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -5765,7 +5765,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -5800,7 +5800,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -5835,7 +5835,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -5870,7 +5870,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -5905,7 +5905,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -5940,7 +5940,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -5975,7 +5975,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -6010,7 +6010,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -6045,7 +6045,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -6080,7 +6080,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -6115,7 +6115,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -6150,7 +6150,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -6185,7 +6185,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -6220,7 +6220,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -6255,7 +6255,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -6290,7 +6290,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -6325,7 +6325,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -6360,7 +6360,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -6395,7 +6395,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -6430,7 +6430,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -6465,7 +6465,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -6500,7 +6500,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -6535,7 +6535,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -6570,7 +6570,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -6605,7 +6605,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -6640,7 +6640,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -6675,7 +6675,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -6710,7 +6710,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -6745,7 +6745,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Riverfront Stadium (Equity Bank Park), 275 S McLean Blvd, Wichita, KS 67213</t>
+          <t>Equity Bank Park, 275 S McLean Blvd, Wichita, KS 67213</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">

</xml_diff>